<commit_message>
Exportación de excel corregida
</commit_message>
<xml_diff>
--- a/Plantilla generación de proformas.xlsx
+++ b/Plantilla generación de proformas.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fslincango\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fslincango\Desktop\CONSTRUMETRICA\Construproformas 2.1\ConstruProformas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E5F3E92-A048-4487-8D12-AC8728E505BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{097B6DE4-D02B-4612-8D04-03DDCD995247}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Planilla" sheetId="10" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Planilla!$A$2:$G$32</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Planilla!$A$2:$G$33</definedName>
     <definedName name="CODIGO">#REF!</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Planilla!$1:$9</definedName>
   </definedNames>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="39">
   <si>
     <t>UNIDAD</t>
   </si>
@@ -150,6 +150,9 @@
   </si>
   <si>
     <t>NOMBRE DEL RUBRO</t>
+  </si>
+  <si>
+    <t>FECHA:</t>
   </si>
 </sst>
 </file>
@@ -252,6 +255,7 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -612,7 +616,7 @@
     </xf>
     <xf numFmtId="44" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -727,80 +731,144 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="17" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="17" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="17" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="20" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="17" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="17" fillId="2" borderId="12" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="13" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="12" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="21" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="17" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="17" fillId="2" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="17" fillId="2" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="17" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -812,96 +880,35 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="17" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="17" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="17" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="4" fontId="21" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="9" fontId="17" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="20" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="17" fillId="2" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="17" fillId="2" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="17" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="17" fillId="2" borderId="12" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="13" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="12" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="17" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -984,13 +991,13 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>938991</xdr:colOff>
-      <xdr:row>20</xdr:row>
+      <xdr:row>21</xdr:row>
       <xdr:rowOff>146537</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>6</xdr:col>
       <xdr:colOff>810841</xdr:colOff>
-      <xdr:row>31</xdr:row>
+      <xdr:row>32</xdr:row>
       <xdr:rowOff>9016</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
@@ -1377,8 +1384,8 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M32"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5"/>
+  <dimension ref="A1:M33"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="15.5"/>
   <cols>
     <col min="1" max="1" width="17.26953125" style="1" customWidth="1"/>
     <col min="2" max="2" width="65.81640625" style="1" customWidth="1"/>
@@ -1394,94 +1401,94 @@
       <c r="A1" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="75" t="s">
         <v>31</v>
       </c>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
+      <c r="C1" s="75"/>
+      <c r="D1" s="75"/>
+      <c r="E1" s="75"/>
       <c r="F1" s="12"/>
       <c r="G1" s="13"/>
     </row>
     <row r="2" spans="1:13" ht="32.25" customHeight="1">
-      <c r="A2" s="82" t="s">
+      <c r="A2" s="76" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="83"/>
-      <c r="C2" s="83"/>
-      <c r="D2" s="83"/>
-      <c r="E2" s="83"/>
-      <c r="F2" s="83"/>
-      <c r="G2" s="84"/>
+      <c r="B2" s="77"/>
+      <c r="C2" s="77"/>
+      <c r="D2" s="77"/>
+      <c r="E2" s="77"/>
+      <c r="F2" s="77"/>
+      <c r="G2" s="78"/>
     </row>
     <row r="3" spans="1:13" ht="24" customHeight="1">
-      <c r="A3" s="88" t="s">
+      <c r="A3" s="68" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="86" t="s">
+      <c r="B3" s="66" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="89" t="s">
+      <c r="C3" s="69" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="89"/>
-      <c r="E3" s="90">
+      <c r="D3" s="69"/>
+      <c r="E3" s="79">
         <v>1793134424001</v>
       </c>
-      <c r="F3" s="90"/>
-      <c r="G3" s="91"/>
+      <c r="F3" s="79"/>
+      <c r="G3" s="80"/>
     </row>
     <row r="4" spans="1:13" ht="18.75" customHeight="1">
       <c r="A4" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="85"/>
-      <c r="C4" s="85" t="s">
+      <c r="B4" s="65"/>
+      <c r="C4" s="65" t="s">
         <v>32</v>
       </c>
-      <c r="D4" s="85"/>
-      <c r="E4" s="85"/>
-      <c r="F4" s="85"/>
-      <c r="G4" s="87"/>
+      <c r="D4" s="65"/>
+      <c r="E4" s="65"/>
+      <c r="F4" s="65"/>
+      <c r="G4" s="67"/>
     </row>
     <row r="5" spans="1:13" ht="23.25" customHeight="1">
       <c r="A5" s="14" t="s">
         <v>12</v>
       </c>
       <c r="B5" s="27"/>
-      <c r="C5" s="67" t="s">
+      <c r="C5" s="81" t="s">
         <v>33</v>
       </c>
-      <c r="D5" s="67"/>
-      <c r="E5" s="67"/>
-      <c r="F5" s="67"/>
-      <c r="G5" s="68"/>
+      <c r="D5" s="81"/>
+      <c r="E5" s="81"/>
+      <c r="F5" s="81"/>
+      <c r="G5" s="82"/>
     </row>
     <row r="6" spans="1:13" ht="18.75" customHeight="1">
       <c r="A6" s="14" t="s">
         <v>13</v>
       </c>
       <c r="B6" s="27"/>
-      <c r="C6" s="69" t="s">
+      <c r="C6" s="83" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="69"/>
-      <c r="E6" s="69"/>
-      <c r="F6" s="70"/>
-      <c r="G6" s="71"/>
+      <c r="D6" s="83"/>
+      <c r="E6" s="83"/>
+      <c r="F6" s="55"/>
+      <c r="G6" s="56"/>
     </row>
     <row r="7" spans="1:13" ht="18.75" customHeight="1">
       <c r="A7" s="14" t="s">
         <v>22</v>
       </c>
       <c r="B7" s="28"/>
-      <c r="C7" s="72" t="s">
+      <c r="C7" s="57" t="s">
         <v>35</v>
       </c>
-      <c r="D7" s="72"/>
-      <c r="E7" s="72"/>
-      <c r="F7" s="72"/>
-      <c r="G7" s="73"/>
+      <c r="D7" s="57"/>
+      <c r="E7" s="57"/>
+      <c r="F7" s="57"/>
+      <c r="G7" s="58"/>
     </row>
     <row r="8" spans="1:13" ht="15.75" customHeight="1">
       <c r="A8" s="14" t="s">
@@ -1489,199 +1496,203 @@
       </c>
       <c r="B8" s="28"/>
       <c r="C8" s="74">
-        <f>+G16</f>
+        <f>+G17</f>
         <v>0</v>
       </c>
       <c r="D8" s="74"/>
       <c r="E8" s="74"/>
-      <c r="F8" s="75"/>
-      <c r="G8" s="76"/>
+      <c r="F8" s="59"/>
+      <c r="G8" s="60"/>
     </row>
     <row r="9" spans="1:13" ht="15.75" customHeight="1">
       <c r="A9" s="14" t="s">
         <v>19</v>
       </c>
       <c r="B9" s="29"/>
-      <c r="C9" s="77" t="str">
-        <f>C15&amp;" "&amp;"Días Calendario"</f>
+      <c r="C9" s="87" t="str">
+        <f>C16&amp;" "&amp;"Días Calendario"</f>
         <v>0 Días Calendario</v>
       </c>
-      <c r="D9" s="77"/>
-      <c r="E9" s="77"/>
-      <c r="F9" s="56"/>
-      <c r="G9" s="78"/>
-    </row>
-    <row r="10" spans="1:13" ht="15" thickBot="1">
-      <c r="A10" s="2"/>
-      <c r="B10" s="30"/>
-      <c r="C10" s="79"/>
-      <c r="D10" s="79"/>
-      <c r="E10" s="80"/>
-      <c r="F10" s="80"/>
-      <c r="G10" s="81"/>
-    </row>
-    <row r="11" spans="1:13" ht="18" customHeight="1" thickTop="1">
-      <c r="A11" s="38" t="s">
+      <c r="D9" s="87"/>
+      <c r="E9" s="87"/>
+      <c r="F9" s="47"/>
+      <c r="G9" s="61"/>
+    </row>
+    <row r="10" spans="1:13" ht="15.75" customHeight="1">
+      <c r="A10" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="29"/>
+      <c r="C10" s="96">
+        <v>46251</v>
+      </c>
+      <c r="D10" s="87"/>
+      <c r="E10" s="87"/>
+      <c r="F10" s="47"/>
+      <c r="G10" s="61"/>
+    </row>
+    <row r="11" spans="1:13" ht="16" thickBot="1">
+      <c r="A11" s="2"/>
+      <c r="B11" s="30"/>
+      <c r="C11" s="62"/>
+      <c r="D11" s="62"/>
+      <c r="E11" s="63"/>
+      <c r="F11" s="63"/>
+      <c r="G11" s="64"/>
+    </row>
+    <row r="12" spans="1:13" ht="18" customHeight="1" thickTop="1">
+      <c r="A12" s="88" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="40" t="s">
+      <c r="B12" s="90" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="34" t="s">
+      <c r="C12" s="34" t="s">
         <v>14</v>
       </c>
-      <c r="D11" s="40" t="s">
+      <c r="D12" s="90" t="s">
         <v>0</v>
       </c>
-      <c r="E11" s="40" t="s">
+      <c r="E12" s="90" t="s">
         <v>4</v>
       </c>
-      <c r="F11" s="40"/>
-      <c r="G11" s="42"/>
-    </row>
-    <row r="12" spans="1:13" ht="15" customHeight="1">
-      <c r="A12" s="39"/>
-      <c r="B12" s="41"/>
-      <c r="C12" s="35" t="s">
+      <c r="F12" s="90"/>
+      <c r="G12" s="92"/>
+    </row>
+    <row r="13" spans="1:13" ht="15" customHeight="1">
+      <c r="A13" s="89"/>
+      <c r="B13" s="91"/>
+      <c r="C13" s="35" t="s">
         <v>16</v>
       </c>
-      <c r="D12" s="41"/>
-      <c r="E12" s="35" t="s">
+      <c r="D13" s="91"/>
+      <c r="E13" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="F12" s="35" t="s">
+      <c r="F13" s="35" t="s">
         <v>26</v>
       </c>
-      <c r="G12" s="36" t="s">
+      <c r="G13" s="36" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="16">
-      <c r="A13" s="43" t="s">
+    <row r="14" spans="1:13" ht="16">
+      <c r="A14" s="93" t="s">
         <v>36</v>
       </c>
-      <c r="B13" s="44"/>
-      <c r="C13" s="44"/>
-      <c r="D13" s="44"/>
-      <c r="E13" s="44"/>
-      <c r="F13" s="44"/>
-      <c r="G13" s="45"/>
-    </row>
-    <row r="14" spans="1:13" ht="53.25" customHeight="1">
-      <c r="A14" s="48" t="s">
+      <c r="B14" s="94"/>
+      <c r="C14" s="94"/>
+      <c r="D14" s="94"/>
+      <c r="E14" s="94"/>
+      <c r="F14" s="94"/>
+      <c r="G14" s="95"/>
+    </row>
+    <row r="15" spans="1:13" ht="53.25" customHeight="1">
+      <c r="A15" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="B14" s="47" t="s">
+      <c r="B15" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="49"/>
-      <c r="D14" s="50"/>
-      <c r="E14" s="51"/>
-      <c r="F14" s="92"/>
-      <c r="G14" s="93"/>
-      <c r="H14" s="37"/>
-    </row>
-    <row r="15" spans="1:13" ht="16">
-      <c r="A15" s="15"/>
-      <c r="B15" s="22" t="s">
+      <c r="C15" s="40"/>
+      <c r="D15" s="41"/>
+      <c r="E15" s="42"/>
+      <c r="F15" s="70"/>
+      <c r="G15" s="71"/>
+      <c r="H15" s="37"/>
+    </row>
+    <row r="16" spans="1:13" ht="16">
+      <c r="A16" s="15"/>
+      <c r="B16" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="66">
-        <f>SUM(C14:C14)</f>
+      <c r="C16" s="54">
+        <f>SUM(C15:C15)</f>
         <v>0</v>
       </c>
-      <c r="D15" s="25"/>
-      <c r="E15" s="26"/>
-      <c r="G15" s="62"/>
-      <c r="M15" s="1" t="s">
+      <c r="D16" s="25"/>
+      <c r="E16" s="26"/>
+      <c r="G16" s="53"/>
+      <c r="M16" s="1" t="s">
         <v>27</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" ht="16">
-      <c r="A16" s="2"/>
-      <c r="F16" s="31" t="s">
-        <v>25</v>
-      </c>
-      <c r="G16" s="94">
-        <f>SUM(G14:G14)</f>
-        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="16">
       <c r="A17" s="2"/>
       <c r="F17" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="G17" s="72">
+        <f>SUM(G15:G15)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="16">
+      <c r="A18" s="2"/>
+      <c r="F18" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="G17" s="94">
-        <f>0.15*G16</f>
+      <c r="G18" s="72">
+        <f>0.15*G17</f>
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="10.5" customHeight="1">
-      <c r="A18" s="2"/>
-      <c r="F18" s="32" t="s">
+    <row r="19" spans="1:7" ht="10.5" customHeight="1">
+      <c r="A19" s="2"/>
+      <c r="F19" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="G18" s="95">
-        <f>+G17+G16</f>
+      <c r="G19" s="73">
+        <f>+G18+G17</f>
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="16">
-      <c r="A19" s="5" t="s">
+    <row r="20" spans="1:7" ht="16">
+      <c r="A20" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B19" s="7"/>
-      <c r="C19" s="33"/>
-      <c r="D19" s="33"/>
-      <c r="E19" s="33"/>
-      <c r="F19" s="32"/>
-      <c r="G19" s="24"/>
-    </row>
-    <row r="20" spans="1:7">
-      <c r="A20" s="60"/>
-      <c r="B20" s="61"/>
-      <c r="C20" s="61"/>
-      <c r="D20" s="61"/>
-      <c r="E20" s="61"/>
-      <c r="F20" s="61"/>
-      <c r="G20" s="62"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="33"/>
+      <c r="D20" s="33"/>
+      <c r="E20" s="33"/>
+      <c r="F20" s="32"/>
+      <c r="G20" s="24"/>
     </row>
     <row r="21" spans="1:7">
-      <c r="A21" s="60"/>
-      <c r="B21" s="61"/>
-      <c r="C21" s="61"/>
-      <c r="D21" s="61"/>
-      <c r="E21" s="61"/>
-      <c r="F21" s="61"/>
-      <c r="G21" s="62"/>
+      <c r="A21" s="51"/>
+      <c r="B21" s="52"/>
+      <c r="C21" s="52"/>
+      <c r="D21" s="52"/>
+      <c r="E21" s="52"/>
+      <c r="F21" s="52"/>
+      <c r="G21" s="53"/>
     </row>
     <row r="22" spans="1:7">
-      <c r="A22" s="63"/>
-      <c r="B22" s="64"/>
-      <c r="C22" s="64"/>
-      <c r="D22" s="64"/>
-      <c r="E22" s="64"/>
-      <c r="F22" s="64"/>
-      <c r="G22" s="65"/>
-    </row>
-    <row r="23" spans="1:7" ht="15.5">
-      <c r="A23" s="52"/>
-      <c r="B23" s="53"/>
-      <c r="C23" s="53"/>
-      <c r="D23" s="53"/>
-      <c r="E23" s="53"/>
-      <c r="F23" s="53"/>
-      <c r="G23" s="54"/>
+      <c r="A22" s="51"/>
+      <c r="B22" s="52"/>
+      <c r="C22" s="52"/>
+      <c r="D22" s="52"/>
+      <c r="E22" s="52"/>
+      <c r="F22" s="52"/>
+      <c r="G22" s="53"/>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" s="84"/>
+      <c r="B23" s="85"/>
+      <c r="C23" s="85"/>
+      <c r="D23" s="85"/>
+      <c r="E23" s="85"/>
+      <c r="F23" s="85"/>
+      <c r="G23" s="86"/>
     </row>
     <row r="24" spans="1:7">
-      <c r="A24" s="18"/>
-      <c r="B24" s="19"/>
-      <c r="C24" s="19"/>
-      <c r="D24" s="19"/>
-      <c r="E24" s="19"/>
-      <c r="F24" s="19"/>
-      <c r="G24" s="20"/>
+      <c r="A24" s="43"/>
+      <c r="B24" s="44"/>
+      <c r="C24" s="44"/>
+      <c r="D24" s="44"/>
+      <c r="E24" s="44"/>
+      <c r="F24" s="44"/>
+      <c r="G24" s="45"/>
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="18"/>
@@ -1710,22 +1721,18 @@
       <c r="F27" s="19"/>
       <c r="G27" s="20"/>
     </row>
-    <row r="28" spans="1:7" ht="15.5">
-      <c r="A28" s="21"/>
-      <c r="B28" s="55"/>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
-      <c r="G28" s="17"/>
-    </row>
-    <row r="29" spans="1:7" ht="16">
-      <c r="A29" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B29" s="56" t="s">
-        <v>21</v>
-      </c>
+    <row r="28" spans="1:7">
+      <c r="A28" s="18"/>
+      <c r="B28" s="19"/>
+      <c r="C28" s="19"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="19"/>
+      <c r="F28" s="19"/>
+      <c r="G28" s="20"/>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" s="21"/>
+      <c r="B29" s="46"/>
       <c r="C29" s="16"/>
       <c r="D29" s="16"/>
       <c r="E29" s="16"/>
@@ -1733,9 +1740,11 @@
       <c r="G29" s="17"/>
     </row>
     <row r="30" spans="1:7" ht="16">
-      <c r="A30" s="8"/>
-      <c r="B30" s="59" t="s">
-        <v>18</v>
+      <c r="A30" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B30" s="47" t="s">
+        <v>21</v>
       </c>
       <c r="C30" s="16"/>
       <c r="D30" s="16"/>
@@ -1743,50 +1752,62 @@
       <c r="F30" s="16"/>
       <c r="G30" s="17"/>
     </row>
-    <row r="31" spans="1:7" ht="15.5">
-      <c r="A31" s="3"/>
-      <c r="B31" s="57" t="s">
+    <row r="31" spans="1:7" ht="16">
+      <c r="A31" s="8"/>
+      <c r="B31" s="50" t="s">
+        <v>18</v>
+      </c>
+      <c r="C31" s="16"/>
+      <c r="D31" s="16"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="16"/>
+      <c r="G31" s="17"/>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32" s="3"/>
+      <c r="B32" s="48" t="s">
         <v>28</v>
       </c>
-      <c r="C31" s="4"/>
-      <c r="D31" s="4"/>
-      <c r="E31" s="4"/>
-      <c r="F31" s="4"/>
-      <c r="G31" s="6"/>
-    </row>
-    <row r="32" spans="1:7" ht="16" thickBot="1">
-      <c r="A32" s="9"/>
-      <c r="B32" s="58" t="s">
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4"/>
+      <c r="F32" s="4"/>
+      <c r="G32" s="6"/>
+    </row>
+    <row r="33" spans="1:7" ht="16" thickBot="1">
+      <c r="A33" s="9"/>
+      <c r="B33" s="49" t="s">
         <v>29</v>
       </c>
-      <c r="C32" s="10"/>
-      <c r="D32" s="10"/>
-      <c r="E32" s="10"/>
-      <c r="F32" s="10"/>
-      <c r="G32" s="11"/>
+      <c r="C33" s="10"/>
+      <c r="D33" s="10"/>
+      <c r="E33" s="10"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
+    <mergeCell ref="A23:G23"/>
+    <mergeCell ref="C9:E9"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="D12:D13"/>
+    <mergeCell ref="E12:G12"/>
+    <mergeCell ref="A14:G14"/>
+    <mergeCell ref="C10:E10"/>
     <mergeCell ref="C8:E8"/>
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="E3:G3"/>
     <mergeCell ref="C5:G5"/>
     <mergeCell ref="C6:E6"/>
-    <mergeCell ref="A22:G22"/>
-    <mergeCell ref="C9:E9"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:G11"/>
-    <mergeCell ref="A13:G13"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.23622047244094488" right="0.23622047244094488" top="0.28000000000000003" bottom="4.68" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="51" orientation="portrait" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
   <ignoredErrors>
-    <ignoredError sqref="C15" emptyCellReference="1"/>
+    <ignoredError sqref="C16" emptyCellReference="1"/>
   </ignoredErrors>
   <drawing r:id="rId2"/>
 </worksheet>

</xml_diff>